<commit_message>
netlify app - submittable form page integrated
</commit_message>
<xml_diff>
--- a/checkouts.xlsx
+++ b/checkouts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,8 +517,38 @@
           <t>2026-06-06 11:09:18</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-06-06 12:34:39</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>